<commit_message>
favicon fixed for serp
</commit_message>
<xml_diff>
--- a/outputs/backlink-created-details.xlsx
+++ b/outputs/backlink-created-details.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
@@ -516,6 +516,210 @@
         </is>
       </c>
       <c r="B8" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>https://www.lapastory.com/guest-posting-canada/</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>https://lendingarch.ca/blog/lendingarch-we-invite-you-to-write-for-us/</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>https://covermove.com/write-for-us/</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>https://www.allaroundmoving.com/write-for-us/</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>https://khabarbandhan.in/write-for-us/</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>https://knowledgeborder.com/write-for-us/</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>https://www.betterplaceimmigration.com/write-for-us/</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>https://themuslimvibe.com/write</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>https://travelwarm.com/write-for-us/</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>https://theoffersguy.com/write-for-us/</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>https://www.99list.ca/submit-guest-post-for-property-car-jobs.html</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>https://lawbhoomi.com/write-for-us-immigration/</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>https://policyoptions.irpp.org/about/article-submission/</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>https://relocationecosystem.com/contribute/</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>https://outcomecanada.ca/submit</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>https://www.vietfederation.ca/write-for-us/</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>https://immigrantmuse.ca/contact-us/</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
         </is>

</xml_diff>

<commit_message>
dark screen in tab and mobile fixed and pankaj khanna rcic number and details added
</commit_message>
<xml_diff>
--- a/outputs/backlink-created-details.xlsx
+++ b/outputs/backlink-created-details.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
@@ -722,6 +722,30 @@
       <c r="B25" t="inlineStr">
         <is>
           <t>https://commonwealthmigration.ca/immigrate/express-entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>https://opencanada.org/open-canada-author-writing-guide/</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/inadmissibility-and-appeals/misrepresentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>https://spheresofinfluence.ca/guest-submissions/</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://commonwealthmigration.ca/sponsor/spousal-and-partner-sponsorship-overview</t>
         </is>
       </c>
     </row>

</xml_diff>